<commit_message>
Modify the thesis tracker excel file
</commit_message>
<xml_diff>
--- a/plan/Thesis_Tracker_10_Weeks_EN.xlsx
+++ b/plan/Thesis_Tracker_10_Weeks_EN.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bernstein/Library/Mobile Documents/com~apple~CloudDocs/Studium/BachelorArbeit/plan/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E9749E2-9F4C-8A44-A880-9E3F94B728D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{192FC8FF-25F4-2B41-9329-65FEC3B4607D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4360" yWindow="660" windowWidth="25840" windowHeight="21680" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
     <sheet name="Weekly Plan" sheetId="2" r:id="rId2"/>
     <sheet name="Checklist" sheetId="3" r:id="rId3"/>
+    <sheet name="Week1" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -30,15 +31,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="150">
   <si>
     <t>Bachelor's Thesis Timeline — 10-Week Tracker</t>
   </si>
@@ -49,13 +47,13 @@
     <t>Official processing time</t>
   </si>
   <si>
-    <t>15 June 2026 – 23 August 2026 (10 weeks)</t>
+    <t>16 June 2026 – 25 August 2026 (10 weeks)</t>
   </si>
   <si>
     <t>Preparation phase</t>
   </si>
   <si>
-    <t>until 14 June 2026 (before the official start)</t>
+    <t>until 15 June 2026 (before the official start)</t>
   </si>
   <si>
     <t>Weekly workload</t>
@@ -73,7 +71,7 @@
     <t>Submission deadline</t>
   </si>
   <si>
-    <t>Sunday, 23 August 2026 at the latest</t>
+    <t>Monday, 25 August 2026 at the latest</t>
   </si>
   <si>
     <t>Overall progress</t>
@@ -231,7 +229,7 @@
     <t>Week 1</t>
   </si>
   <si>
-    <t>15–21 Jun</t>
+    <t>15–22 Jun</t>
   </si>
   <si>
     <t>Literature review &amp; consolidating PyTorch</t>
@@ -240,7 +238,7 @@
     <t>Week 2</t>
   </si>
   <si>
-    <t>22–28 Jun</t>
+    <t>22–29 Jun</t>
   </si>
   <si>
     <t>Fixing the method &amp; drafting Related Work</t>
@@ -258,7 +256,7 @@
     <t>Week 4</t>
   </si>
   <si>
-    <t>6–12 Jul</t>
+    <t>6–13 Jul</t>
   </si>
   <si>
     <t>Contrastive training &amp; first end-to-end pipeline</t>
@@ -285,7 +283,7 @@
     <t>Week 7</t>
   </si>
   <si>
-    <t>27 Jul–2 Aug</t>
+    <t>27 Jul–3 Aug</t>
   </si>
   <si>
     <t>Sensitivity studies &amp; failure cases</t>
@@ -303,7 +301,7 @@
     <t>Week 9</t>
   </si>
   <si>
-    <t>10–16 Aug</t>
+    <t>10–17 Aug</t>
   </si>
   <si>
     <t>Discussion &amp; complete first draft</t>
@@ -312,7 +310,7 @@
     <t>Week 10</t>
   </si>
   <si>
-    <t>17–23 Aug</t>
+    <t>17–25 Aug</t>
   </si>
   <si>
     <t>Total</t>
@@ -330,18 +328,21 @@
     <t>Set up the Python environment (Miniconda/venv, Jupyter/VS Code, Git)</t>
   </si>
   <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Learn numpy &amp; pandas: arrays, DataFrames, indexing, loading CSV</t>
+  </si>
+  <si>
+    <t>Learn matplotlib: scatter plots, histograms, learning curves</t>
+  </si>
+  <si>
+    <t>Learn scikit-learn: StandardScaler, KMeans, NMI/ARI/silhouette</t>
+  </si>
+  <si>
     <t>No</t>
   </si>
   <si>
-    <t>Learn numpy &amp; pandas: arrays, DataFrames, indexing, loading CSV</t>
-  </si>
-  <si>
-    <t>Learn matplotlib: scatter plots, histograms, learning curves</t>
-  </si>
-  <si>
-    <t>Learn scikit-learn: StandardScaler, KMeans, NMI/ARI/silhouette</t>
-  </si>
-  <si>
     <t>Mini-project: cluster Iris/Digits, compute NMI/ARI, plot embedding</t>
   </si>
   <si>
@@ -375,6 +376,9 @@
     <t>Select 3–4 tabular datasets with ground-truth labels</t>
   </si>
   <si>
+    <t>Classify each dataset by feature type: fraction of categorical vs. numerical features; identify features with highest mutual information with cluster labels</t>
+  </si>
+  <si>
     <t>Define the structure; write the related-work draft</t>
   </si>
   <si>
@@ -387,6 +391,9 @@
     <t>Augmentation module scaffold: feature masking/corruption (SCARF)</t>
   </si>
   <si>
+    <t>Implement feature-type mask: categorical → marginal-distribution replacement; numerical → Gaussian noise or scaling</t>
+  </si>
+  <si>
     <t>Implement the encoder network (MLP)</t>
   </si>
   <si>
@@ -405,6 +412,12 @@
     <t>Further augmentations: Gaussian noise, feature swapping, zeroing/mixup</t>
   </si>
   <si>
+    <t>Add no-augmentation baseline: identity augmentation (each row passed twice unchanged); label "Identity" in all result tables</t>
+  </si>
+  <si>
+    <t>Add feature-type-aware pipeline as a fourth technique; label "Type-Aware" in all result tables</t>
+  </si>
+  <si>
     <t>Reproducibility: seeds, configuration files, CSV logging</t>
   </si>
   <si>
@@ -429,25 +442,31 @@
     <t>Investigate limitations and failure cases</t>
   </si>
   <si>
+    <t>Produce stratified results tables: NMI and ARI broken down by dataset taxonomy (&gt;50% categorical vs. mostly numerical)</t>
+  </si>
+  <si>
     <t>Prepare results as tables and figures</t>
   </si>
   <si>
     <t>Supervisor meeting: discuss the results</t>
   </si>
   <si>
-    <t>Analyse results: which augmentation helps/hurts</t>
-  </si>
-  <si>
-    <t>Write the “Methodology” chapter (LaTeX)</t>
-  </si>
-  <si>
-    <t>Write the “Experiments &amp; Results” chapter</t>
-  </si>
-  <si>
-    <t>Write the “Discussion” chapter</t>
-  </si>
-  <si>
-    <t>Write introduction, related work, conclusion &amp; outlook, abstract</t>
+    <t>Analyse results: which augmentation helps/hurts and why</t>
+  </si>
+  <si>
+    <t>Analyse stratified results: Identity baseline vs. augmented variants on high-categorical datasets; Type-Aware pipeline improvement</t>
+  </si>
+  <si>
+    <t>Write the "Methodology" chapter (LaTeX)</t>
+  </si>
+  <si>
+    <t>Write the "Experiments &amp; Results" chapter</t>
+  </si>
+  <si>
+    <t>Write the "Discussion" chapter: interpretation, contextualisation, limitations</t>
+  </si>
+  <si>
+    <t>Write introduction, related work (finalise), conclusion &amp; outlook, abstract</t>
   </si>
   <si>
     <t>Merge the full document, hand it to the supervisor</t>
@@ -468,7 +487,16 @@
     <t>Buffer for unforeseen issues</t>
   </si>
   <si>
-    <t>Yes</t>
+    <t>In progress</t>
+  </si>
+  <si>
+    <t>Until Sunday 22.06</t>
+  </si>
+  <si>
+    <t>Learn Pytorch</t>
+  </si>
+  <si>
+    <t>Skim survey</t>
   </si>
 </sst>
 </file>
@@ -476,8 +504,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="0&quot; h&quot;"/>
+    <numFmt numFmtId="164" formatCode="0&quot; h&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -677,7 +705,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -743,7 +771,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -752,28 +780,29 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1117,146 +1146,146 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
-      <c r="J2" s="39"/>
-      <c r="K2" s="39"/>
-      <c r="L2" s="39"/>
-      <c r="M2" s="39"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37" t="s">
+      <c r="B4" s="32"/>
+      <c r="C4" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="37"/>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
-      <c r="H4" s="37"/>
-      <c r="I4" s="37"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="37" t="s">
+      <c r="B5" s="32"/>
+      <c r="C5" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="36"/>
-      <c r="C6" s="37" t="s">
+      <c r="B6" s="32"/>
+      <c r="C6" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="37"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="36"/>
-      <c r="C7" s="37" t="s">
+      <c r="B7" s="32"/>
+      <c r="C7" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="36"/>
-      <c r="C8" s="37" t="s">
+      <c r="B8" s="32"/>
+      <c r="C8" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37"/>
-      <c r="I8" s="37"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="38" t="s">
         <v>12</v>
       </c>
       <c r="B9" s="32"/>
-      <c r="C9" s="33">
-        <f>COUNTIF(Checklist!D4:D49,"Yes")/46</f>
-        <v>6.5217391304347824E-2</v>
-      </c>
-      <c r="D9" s="33"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
-    </row>
-    <row r="11" spans="1:13" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="34" t="s">
+      <c r="C9" s="34">
+        <f>COUNTIF(Checklist!D4:D55,"Yes")/52</f>
+        <v>7.6923076923076927E-2</v>
+      </c>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
+    </row>
+    <row r="11" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="34"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="34"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="34"/>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
-      <c r="M11" s="34"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="32"/>
+      <c r="L11" s="32"/>
+      <c r="M11" s="32"/>
     </row>
     <row r="12" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
@@ -1445,40 +1474,40 @@
       </c>
     </row>
     <row r="21" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="35" t="s">
+      <c r="A21" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="B21" s="35"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35"/>
-      <c r="G21" s="35"/>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35"/>
-      <c r="J21" s="35"/>
-      <c r="K21" s="35"/>
-      <c r="L21" s="35"/>
-      <c r="M21" s="35"/>
+      <c r="B21" s="32"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+      <c r="L21" s="32"/>
+      <c r="M21" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A21:M21"/>
+    <mergeCell ref="C6:I6"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A11:M11"/>
+    <mergeCell ref="C9:I9"/>
     <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C8:I8"/>
     <mergeCell ref="C4:I4"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A2:M2"/>
     <mergeCell ref="C5:I5"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:I9"/>
-    <mergeCell ref="A11:M11"/>
-    <mergeCell ref="A21:M21"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:I6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:I8"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1505,16 +1534,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="40" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
     </row>
     <row r="3" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
@@ -1557,11 +1586,11 @@
       </c>
       <c r="E4" s="22"/>
       <c r="F4" s="22" t="str">
-        <f>COUNTIFS(Checklist!$A$4:$A$49,0,Checklist!$D$4:$D$49,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$49,0)</f>
+        <f>COUNTIFS(Checklist!$A$4:$A$55,0,Checklist!$D$4:$D$55,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$55,0)</f>
         <v>3 / 7</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>58</v>
+        <v>91</v>
       </c>
       <c r="H4" s="22"/>
     </row>
@@ -1582,11 +1611,11 @@
         <v>22</v>
       </c>
       <c r="F5" s="25" t="str">
-        <f>COUNTIFS(Checklist!$A$4:$A$49,1,Checklist!$D$4:$D$49,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$49,1)</f>
-        <v>0 / 6</v>
+        <f>COUNTIFS(Checklist!$A$4:$A$55,1,Checklist!$D$4:$D$55,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$55,1)</f>
+        <v>1 / 6</v>
       </c>
       <c r="G5" s="25" t="s">
-        <v>58</v>
+        <v>146</v>
       </c>
       <c r="H5" s="28" t="s">
         <v>41</v>
@@ -1609,8 +1638,8 @@
         <v>22</v>
       </c>
       <c r="F6" s="25" t="str">
-        <f>COUNTIFS(Checklist!$A$4:$A$49,2,Checklist!$D$4:$D$49,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$49,2)</f>
-        <v>0 / 4</v>
+        <f>COUNTIFS(Checklist!$A$4:$A$55,2,Checklist!$D$4:$D$55,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$55,2)</f>
+        <v>0 / 5</v>
       </c>
       <c r="G6" s="25" t="s">
         <v>58</v>
@@ -1636,8 +1665,8 @@
         <v>22</v>
       </c>
       <c r="F7" s="25" t="str">
-        <f>COUNTIFS(Checklist!$A$4:$A$49,3,Checklist!$D$4:$D$49,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$49,3)</f>
-        <v>0 / 3</v>
+        <f>COUNTIFS(Checklist!$A$4:$A$55,3,Checklist!$D$4:$D$55,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$55,3)</f>
+        <v>0 / 4</v>
       </c>
       <c r="G7" s="25" t="s">
         <v>58</v>
@@ -1661,7 +1690,7 @@
         <v>22</v>
       </c>
       <c r="F8" s="25" t="str">
-        <f>COUNTIFS(Checklist!$A$4:$A$49,4,Checklist!$D$4:$D$49,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$49,4)</f>
+        <f>COUNTIFS(Checklist!$A$4:$A$55,4,Checklist!$D$4:$D$55,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$55,4)</f>
         <v>0 / 4</v>
       </c>
       <c r="G8" s="25" t="s">
@@ -1688,8 +1717,8 @@
         <v>22</v>
       </c>
       <c r="F9" s="25" t="str">
-        <f>COUNTIFS(Checklist!$A$4:$A$49,5,Checklist!$D$4:$D$49,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$49,5)</f>
-        <v>0 / 4</v>
+        <f>COUNTIFS(Checklist!$A$4:$A$55,5,Checklist!$D$4:$D$55,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$55,5)</f>
+        <v>0 / 6</v>
       </c>
       <c r="G9" s="25" t="s">
         <v>58</v>
@@ -1713,7 +1742,7 @@
         <v>22</v>
       </c>
       <c r="F10" s="25" t="str">
-        <f>COUNTIFS(Checklist!$A$4:$A$49,6,Checklist!$D$4:$D$49,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$49,6)</f>
+        <f>COUNTIFS(Checklist!$A$4:$A$55,6,Checklist!$D$4:$D$55,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$55,6)</f>
         <v>0 / 3</v>
       </c>
       <c r="G10" s="25" t="s">
@@ -1738,8 +1767,8 @@
         <v>22</v>
       </c>
       <c r="F11" s="25" t="str">
-        <f>COUNTIFS(Checklist!$A$4:$A$49,7,Checklist!$D$4:$D$49,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$49,7)</f>
-        <v>0 / 4</v>
+        <f>COUNTIFS(Checklist!$A$4:$A$55,7,Checklist!$D$4:$D$55,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$55,7)</f>
+        <v>0 / 5</v>
       </c>
       <c r="G11" s="25" t="s">
         <v>58</v>
@@ -1765,8 +1794,8 @@
         <v>22</v>
       </c>
       <c r="F12" s="25" t="str">
-        <f>COUNTIFS(Checklist!$A$4:$A$49,8,Checklist!$D$4:$D$49,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$49,8)</f>
-        <v>0 / 3</v>
+        <f>COUNTIFS(Checklist!$A$4:$A$55,8,Checklist!$D$4:$D$55,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$55,8)</f>
+        <v>0 / 4</v>
       </c>
       <c r="G12" s="25" t="s">
         <v>58</v>
@@ -1790,7 +1819,7 @@
         <v>22</v>
       </c>
       <c r="F13" s="25" t="str">
-        <f>COUNTIFS(Checklist!$A$4:$A$49,9,Checklist!$D$4:$D$49,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$49,9)</f>
+        <f>COUNTIFS(Checklist!$A$4:$A$55,9,Checklist!$D$4:$D$55,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$55,9)</f>
         <v>0 / 3</v>
       </c>
       <c r="G13" s="25" t="s">
@@ -1817,7 +1846,7 @@
         <v>22</v>
       </c>
       <c r="F14" s="25" t="str">
-        <f>COUNTIFS(Checklist!$A$4:$A$49,10,Checklist!$D$4:$D$49,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$49,10)</f>
+        <f>COUNTIFS(Checklist!$A$4:$A$55,10,Checklist!$D$4:$D$55,"Yes")&amp;" / "&amp;COUNTIF(Checklist!$A$4:$A$55,10)</f>
         <v>0 / 5</v>
       </c>
       <c r="G14" s="25" t="s">
@@ -1868,7 +1897,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="8" customWidth="1"/>
@@ -1877,12 +1906,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="40" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
     </row>
     <row r="3" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
@@ -1909,7 +1938,7 @@
         <v>92</v>
       </c>
       <c r="D4" s="25" t="s">
-        <v>139</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -1923,7 +1952,7 @@
         <v>94</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>139</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -1937,7 +1966,7 @@
         <v>95</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>139</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -1951,7 +1980,7 @@
         <v>96</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -1962,10 +1991,10 @@
         <v>27</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D8" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -1976,10 +2005,10 @@
         <v>27</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D9" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -1990,10 +2019,10 @@
         <v>27</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D10" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -2004,7 +2033,7 @@
         <v>29</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D11" s="25" t="s">
         <v>93</v>
@@ -2018,10 +2047,10 @@
         <v>29</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -2032,10 +2061,10 @@
         <v>29</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -2046,10 +2075,10 @@
         <v>29</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D14" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -2060,10 +2089,10 @@
         <v>29</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D15" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -2074,10 +2103,10 @@
         <v>29</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D16" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -2088,10 +2117,10 @@
         <v>29</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -2102,13 +2131,13 @@
         <v>29</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A19" s="24">
         <v>2</v>
       </c>
@@ -2116,10 +2145,10 @@
         <v>29</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -2130,24 +2159,24 @@
         <v>29</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="24">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -2158,10 +2187,10 @@
         <v>31</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -2172,38 +2201,38 @@
         <v>31</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A24" s="24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B24" s="9" t="s">
         <v>31</v>
       </c>
       <c r="C24" s="26" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D24" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B25" s="9" t="s">
         <v>31</v>
       </c>
       <c r="C25" s="26" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -2214,10 +2243,10 @@
         <v>31</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D26" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -2228,38 +2257,38 @@
         <v>31</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="24">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="9" t="s">
         <v>31</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D28" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="24">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B29" s="9" t="s">
         <v>31</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D29" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -2270,13 +2299,13 @@
         <v>31</v>
       </c>
       <c r="C30" s="26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D30" s="25" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A31" s="24">
         <v>5</v>
       </c>
@@ -2284,262 +2313,346 @@
         <v>31</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D31" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="24">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D32" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="24">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D33" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="24">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C34" s="26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D34" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="24">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D35" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="24">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B36" s="11" t="s">
         <v>33</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D36" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="24">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B37" s="11" t="s">
         <v>33</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D37" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="24">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B38" s="11" t="s">
         <v>33</v>
       </c>
       <c r="C38" s="26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D38" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="24">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C39" s="26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D39" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="24">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C40" s="26" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D40" s="25" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A41" s="24">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D41" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="24">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C42" s="26" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D42" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="24">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C43" s="26" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D43" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="24">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B44" s="13" t="s">
         <v>35</v>
       </c>
       <c r="C44" s="26" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D44" s="25" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A45" s="24">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B45" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C45" s="26" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D45" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="24">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C46" s="26" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D46" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="24">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C47" s="26" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D47" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="24">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C48" s="26" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D48" s="25" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="24">
+        <v>9</v>
+      </c>
+      <c r="B49" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C49" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="D49" s="25" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>9</v>
+      </c>
+      <c r="B50" t="s">
+        <v>35</v>
+      </c>
+      <c r="C50" t="s">
+        <v>140</v>
+      </c>
+      <c r="D50" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51">
         <v>10</v>
       </c>
-      <c r="B49" s="15" t="s">
+      <c r="B51" t="s">
         <v>37</v>
       </c>
-      <c r="C49" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="D49" s="25" t="s">
-        <v>93</v>
+      <c r="C51" t="s">
+        <v>141</v>
+      </c>
+      <c r="D51" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>10</v>
+      </c>
+      <c r="B52" t="s">
+        <v>37</v>
+      </c>
+      <c r="C52" t="s">
+        <v>142</v>
+      </c>
+      <c r="D52" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>10</v>
+      </c>
+      <c r="B53" t="s">
+        <v>37</v>
+      </c>
+      <c r="C53" t="s">
+        <v>143</v>
+      </c>
+      <c r="D53" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>10</v>
+      </c>
+      <c r="B54" t="s">
+        <v>37</v>
+      </c>
+      <c r="C54" t="s">
+        <v>144</v>
+      </c>
+      <c r="D54" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>10</v>
+      </c>
+      <c r="B55" t="s">
+        <v>37</v>
+      </c>
+      <c r="C55" t="s">
+        <v>145</v>
+      </c>
+      <c r="D55" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -2564,4 +2677,38 @@
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToHeight="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5B5010C-C443-884E-9708-45F8083CAAAF}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>